<commit_message>
Migrar documentacion a PHP 8.2 + Laravel 11 + MySQL 8
</commit_message>
<xml_diff>
--- a/_docs_/trim01/04_requisitos/CS_RequistosFuncionales_Matrix_.xlsx
+++ b/_docs_/trim01/04_requisitos/CS_RequistosFuncionales_Matrix_.xlsx
@@ -861,7 +861,7 @@
     <t>Portabilidad</t>
   </si>
   <si>
-    <t>El sistema debe poder ejecutarse en SQLite (ambiente de pruebas) y PostgreSQL (producción) sin requerir cambios en el código fuente. El sistema deberá poder desplegarse en servidores Linux (Ubuntu 22.04) o Windows Server.</t>
+    <t>El sistema debe poder ejecutarse sobre MySQL 8 tanto en ambiente de pruebas como en producción, sin requerir cambios en el código fuente. El sistema deberá poder desplegarse en servidores Linux (Ubuntu 22.04) o Windows Server.</t>
   </si>
   <si>
     <t>RNF09</t>
@@ -870,7 +870,7 @@
     <t>Mantenibilidad</t>
   </si>
   <si>
-    <t>El código fuente del sistema debe estar organizado siguiendo el patrón MTV de Django (Model – Template – View), con comentarios en funciones clave y nombres de variables descriptivos en español. Cada módulo debe estar separado como aplicación Django independiente.</t>
+    <t>El código fuente del sistema debe estar organizado siguiendo el patrón MVC de Laravel (Model – View – Controller), con comentarios en funciones clave y nombres de variables descriptivos en español. Cada módulo debe estar separado con sus propios controladores y modelos independientes.</t>
   </si>
   <si>
     <t>RNF10</t>

</xml_diff>